<commit_message>
release: TSMAI-RC-001 - Release Candidate v1.0.0 for Netlify Staging
PRD-REL001-AUD-R1: Integracion completa de calendarios unificados (PRD-CAL001-R1), reagendamiento trazable (PRD-CAL002-R1), cierre/rechazo de OT (PRD-OT003-R1/R1.1), evidencias fotograficas 360 (PRD-EVI001-R1), SPA redirects en Netlify y verificacion de seguridad RLS.
</commit_message>
<xml_diff>
--- a/importar_excel/LISTADO_SOLICITANTES.xlsx
+++ b/importar_excel/LISTADO_SOLICITANTES.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\franh\OneDrive\Documentos\GuIA\Proyectos\TSMAI\app\importar_excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d6abab3e387e8272/Documentos/GuIA/Proyectos/TSMAI/app/importar_excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BF0C789D-0D21-4C35-BC32-E30CA81BF560}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="8_{BF0C789D-0D21-4C35-BC32-E30CA81BF560}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FFC08344-121B-4CBD-B333-2D8403CF9121}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="900" windowWidth="29040" windowHeight="15720" xr2:uid="{AB654B36-4D20-4D9D-803D-DB6016586B72}"/>
+    <workbookView xWindow="28680" yWindow="1650" windowWidth="29040" windowHeight="15720" xr2:uid="{AB654B36-4D20-4D9D-803D-DB6016586B72}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>

</xml_diff>